<commit_message>
Implemented calculation of crop P requirements
</commit_message>
<xml_diff>
--- a/data/default/Regions.xlsx
+++ b/data/default/Regions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="46">
   <si>
     <t>f_region</t>
   </si>
@@ -143,6 +143,21 @@
   </si>
   <si>
     <t>Lindahl &amp; Lundblad (2021)</t>
+  </si>
+  <si>
+    <t>soil_P_AL</t>
+  </si>
+  <si>
+    <t>soil_K_AL</t>
+  </si>
+  <si>
+    <t>mg/kg</t>
+  </si>
+  <si>
+    <t>soil P-AL concentration</t>
+  </si>
+  <si>
+    <t>soil K-AL concentration</t>
   </si>
 </sst>
 </file>
@@ -500,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -688,83 +703,127 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="2">
-        <v>20</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>27</v>
+      <c r="C14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="2">
-        <v>40</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>28</v>
+      <c r="C15" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C16" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D16" s="2">
-        <v>40</v>
+        <v>20</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C17" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D17" s="2">
-        <v>4.4000000000000004</v>
+        <v>40</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C20" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D20" s="2">
         <v>6.4</v>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C20" s="4" t="s">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D24" t="s">
         <v>32</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E24" t="s">
         <v>13</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F24" t="s">
         <v>37</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G24" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C25" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D25" s="4">
         <v>0</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E25" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
x0_crops as parameter and some new crop types
</commit_message>
<xml_diff>
--- a/data/default/Regions.xlsx
+++ b/data/default/Regions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="49">
   <si>
     <t>f_region</t>
   </si>
@@ -158,6 +158,15 @@
   </si>
   <si>
     <t>soil K-AL concentration</t>
+  </si>
+  <si>
+    <t>Baseline crop areas and animal numbers (x0)</t>
+  </si>
+  <si>
+    <t>x0_crops</t>
+  </si>
+  <si>
+    <t>Regions-x0_crops.csv</t>
   </si>
 </sst>
 </file>
@@ -227,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -235,6 +244,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -515,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -550,7 +560,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -560,270 +570,312 @@
       <c r="G2" s="6"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>17</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="G5" t="s">
-        <v>17</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
-        <v>30</v>
-      </c>
-      <c r="E10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s">
-        <v>23</v>
-      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s">
-        <v>22</v>
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D13" t="s">
         <v>30</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D14" t="s">
         <v>30</v>
       </c>
       <c r="E14" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="F14" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
         <v>30</v>
       </c>
       <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" t="s">
         <v>43</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+      <c r="E19" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C16" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="2">
-        <v>20</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="2">
-        <v>40</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="2">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="2">
-        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C20" s="2" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D20" s="2">
-        <v>6.4</v>
+        <v>20</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C21" s="2" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D21" s="2">
-        <v>77</v>
+        <v>40</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="2">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C25" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C26" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D26" s="2">
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C24" s="4" t="s">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C28" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D28" t="s">
         <v>32</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E28" t="s">
         <v>13</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F28" t="s">
         <v>37</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G28" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C29" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D29" s="4">
         <v>0</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E29" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
x0_animals as parameters + rerun notebooks
</commit_message>
<xml_diff>
--- a/data/default/Regions.xlsx
+++ b/data/default/Regions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
   <si>
     <t>f_region</t>
   </si>
@@ -167,6 +167,12 @@
   </si>
   <si>
     <t>Regions-x0_crops.csv</t>
+  </si>
+  <si>
+    <t>Regions-x0_animals.csv</t>
+  </si>
+  <si>
+    <t>x0_animals</t>
   </si>
 </sst>
 </file>
@@ -585,8 +591,12 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
+      <c r="C4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>49</v>
+      </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>

</xml_diff>